<commit_message>
Updates to hodson analysis
</commit_message>
<xml_diff>
--- a/refs/wart-flights.xlsx
+++ b/refs/wart-flights.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rblack/_projects/mmR2T3/refs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{98B27074-B3D9-2A47-AB8D-1F20A702ED4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D219458-6826-E346-974F-25A363CE8EC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="26240" windowHeight="14660" xr2:uid="{6F3648B4-9E08-B641-B142-5EC1E81BAFE5}"/>
   </bookViews>
@@ -174,12 +174,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -194,7 +200,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -205,6 +211,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2856,75 +2868,75 @@
         <v>1.9170380875202593</v>
       </c>
     </row>
-    <row r="22" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A22">
+    <row r="22" spans="1:27" s="10" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="10">
         <v>2003</v>
       </c>
-      <c r="C22">
+      <c r="C22" s="10">
         <v>47</v>
       </c>
-      <c r="D22">
+      <c r="D22" s="10">
         <v>0.86</v>
       </c>
-      <c r="H22">
+      <c r="H22" s="10">
         <v>18</v>
       </c>
-      <c r="I22">
+      <c r="I22" s="10">
         <v>3660</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="11">
         <f t="shared" si="16"/>
         <v>203.33333333333334</v>
       </c>
-      <c r="K22">
+      <c r="K22" s="10">
         <v>3.1</v>
       </c>
-      <c r="L22" s="3">
+      <c r="L22" s="12">
         <v>10</v>
       </c>
-      <c r="M22">
+      <c r="M22" s="10">
         <v>18</v>
       </c>
-      <c r="N22">
+      <c r="N22" s="10">
         <f t="shared" si="17"/>
         <v>618</v>
       </c>
-      <c r="O22" s="1">
+      <c r="O22" s="13">
         <f t="shared" si="18"/>
         <v>5.9223300970873787</v>
       </c>
-      <c r="Q22" s="2"/>
-      <c r="R22" s="5"/>
-      <c r="S22" s="4"/>
-      <c r="T22" s="5">
+      <c r="Q22" s="11"/>
+      <c r="R22" s="14"/>
+      <c r="S22" s="15"/>
+      <c r="T22" s="14">
         <f t="shared" si="25"/>
         <v>0.72901921132457026</v>
       </c>
-      <c r="U22" s="5">
+      <c r="U22" s="14">
         <f t="shared" si="8"/>
         <v>0.41747572815533979</v>
       </c>
-      <c r="V22" s="1">
+      <c r="V22" s="13">
         <f>6.61 * D22</f>
         <v>5.6846000000000005</v>
       </c>
-      <c r="W22" s="3">
+      <c r="W22" s="12">
         <f t="shared" si="20"/>
         <v>3726.8790106730521</v>
       </c>
-      <c r="X22" s="5">
+      <c r="X22" s="14">
         <f t="shared" si="21"/>
         <v>0.98205495523693587</v>
       </c>
-      <c r="Y22" s="5">
+      <c r="Y22" s="14">
         <f t="shared" si="22"/>
         <v>3.0393442622950819</v>
       </c>
-      <c r="Z22">
+      <c r="Z22" s="10">
         <f t="shared" si="23"/>
         <v>0.12600702334228464</v>
       </c>
-      <c r="AA22">
+      <c r="AA22" s="10">
         <f t="shared" si="24"/>
         <v>1.9104290635765737</v>
       </c>

</xml_diff>